<commit_message>
Finished with local version
</commit_message>
<xml_diff>
--- a/Introtext.xlsx
+++ b/Introtext.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/lucas/Documents/Experiments/Mood4/github_Mood4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DFC8F1DB-155A-B940-8E2D-3C975FE923DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9DECC53-55B9-C34B-BD7E-8676EF668574}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1160" yWindow="760" windowWidth="16780" windowHeight="22840" xr2:uid="{402AE53E-8E8E-A647-AB36-D93CAEC0D9A2}"/>
+    <workbookView xWindow="2980" yWindow="600" windowWidth="41600" windowHeight="22840" xr2:uid="{402AE53E-8E8E-A647-AB36-D93CAEC0D9A2}"/>
   </bookViews>
   <sheets>
     <sheet name="Introtext" sheetId="1" r:id="rId1"/>
@@ -32,12 +32,12 @@
     <t>In the next few steps, we will guide you through the task and how it works, you will then do a minimum of 10 practice trials, and finally, you will start the task.</t>
   </si>
   <si>
-    <t>You will begin the task with $5. The outcome of the choices you make from then on will count for ADDITIONAL money.
-Please select your gamble choice by pressing the LEFT or RIGHT arrow keys. Once you’ve made your choice, the outcome will be applied to your total. 
-On the next screen, you will do a few introductory trials.</t>
+    <t>On each trial, you will have the opportunity to earn money. You will be presented with two options: one option will be a certain reward, the other, a gamble. The gamble probability will be indicated by the percentage number. The gamble has two possible outcomes: either you win and gain the indicated reward, either you lose and earn $0. On some trials, you will only be presented with one option, you will have to selected it.</t>
   </si>
   <si>
-    <t xml:space="preserve">On each trial, you will have the opportunity to earn money. You will be presented with two options: one option will be a certain reward, the other, a gamble. The gamble probability will be indicated by the percentage number. The gamble has two possible outcomes: either you win and gain the indicated reward, either you lose and earn $0. </t>
+    <t>You will begin the task with $5. The outcome of the choices you make from then on will count for ADDITIONAL money.
+Please select your option by pressing the LEFT or RIGHT arrow keys, or either, if you are shown only one option. Once you’ve made your choice, the outcome will be applied to your total. 
+On the next screen, you will do a few introductory trials.</t>
   </si>
 </sst>
 </file>
@@ -934,12 +934,12 @@
     </row>
     <row r="4" spans="1:1" ht="192" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="5" spans="1:1" ht="207" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
   </sheetData>

</xml_diff>